<commit_message>
Add SHELF_PRICE_BOARD so catalog import matches the new sheet (subcategory, sizes, packing, discount) and MRP/discount can be edited on Subcategories and Product Groups as well as Manage Catalog.
Turn off with SHELF_PRICE_BOARD_ENABLED, or delete frontend/src/features/shelf-price-board/ plus those two page imports if the client does not want it.
</commit_message>
<xml_diff>
--- a/frontend/astral-products-import-test.xlsx
+++ b/frontend/astral-products-import-test.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="99">
   <si>
     <t>category</t>
   </si>
@@ -106,6 +106,9 @@
     <t>PIPE SDR-11</t>
   </si>
   <si>
+    <t>4mm</t>
+  </si>
+  <si>
     <t>M511130301</t>
   </si>
   <si>
@@ -115,6 +118,9 @@
     <t>PIPE SDR-13.5</t>
   </si>
   <si>
+    <t>3mm</t>
+  </si>
+  <si>
     <t>M511400307</t>
   </si>
   <si>
@@ -139,6 +145,9 @@
     <t>PIPE CTS SDR 09</t>
   </si>
   <si>
+    <t>2mm</t>
+  </si>
+  <si>
     <t>M511090302</t>
   </si>
   <si>
@@ -149,6 +158,9 @@
   </si>
   <si>
     <t>PIPE SCHEDULE 80</t>
+  </si>
+  <si>
+    <t>1mm</t>
   </si>
   <si>
     <t>M511800507</t>
@@ -798,13 +810,13 @@
         <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G3" t="s">
         <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I3" t="s">
         <v>24</v>
@@ -822,7 +834,7 @@
         <v>18</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P3" t="s">
         <v>28</v>
@@ -839,22 +851,22 @@
         <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
         <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
         <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
         <v>24</v>
@@ -866,13 +878,13 @@
         <v>4875</v>
       </c>
       <c r="L4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N4">
         <v>36</v>
       </c>
       <c r="O4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="P4" t="s">
         <v>28</v>
@@ -889,22 +901,22 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
         <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
         <v>22</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s">
         <v>24</v>
@@ -922,7 +934,7 @@
         <v>94</v>
       </c>
       <c r="O5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P5" t="s">
         <v>28</v>
@@ -939,22 +951,22 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
       </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
         <v>22</v>
       </c>
       <c r="H6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
         <v>24</v>
@@ -972,7 +984,7 @@
         <v>71</v>
       </c>
       <c r="O6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="P6" t="s">
         <v>28</v>
@@ -989,22 +1001,22 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
         <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="G7" t="s">
         <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="I7" t="s">
         <v>24</v>
@@ -1022,7 +1034,7 @@
         <v>36</v>
       </c>
       <c r="O7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P7" t="s">
         <v>28</v>
@@ -1033,28 +1045,28 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
         <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
@@ -1072,10 +1084,10 @@
         <v>99</v>
       </c>
       <c r="O8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="P8" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="Q8" t="s">
         <v>29</v>
@@ -1083,28 +1095,28 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="G9" t="s">
         <v>22</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I9" t="s">
         <v>24</v>
@@ -1122,10 +1134,10 @@
         <v>30</v>
       </c>
       <c r="O9" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="P9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="Q9" t="s">
         <v>29</v>
@@ -1133,28 +1145,28 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="G10" t="s">
         <v>22</v>
       </c>
       <c r="H10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I10" t="s">
         <v>24</v>
@@ -1166,7 +1178,7 @@
         <v>16</v>
       </c>
       <c r="L10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N10">
         <v>86</v>
@@ -1175,7 +1187,7 @@
         <v>27</v>
       </c>
       <c r="P10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="Q10" t="s">
         <v>29</v>
@@ -1183,28 +1195,28 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
         <v>20</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="G11" t="s">
         <v>22</v>
       </c>
       <c r="H11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
         <v>24</v>
@@ -1222,10 +1234,10 @@
         <v>81</v>
       </c>
       <c r="O11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="P11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="Q11" t="s">
         <v>29</v>
@@ -1233,28 +1245,28 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
         <v>20</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
         <v>22</v>
       </c>
       <c r="H12" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
         <v>24</v>
@@ -1272,10 +1284,10 @@
         <v>106</v>
       </c>
       <c r="O12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="P12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Q12" t="s">
         <v>29</v>
@@ -1283,28 +1295,28 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s">
         <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="G13" t="s">
         <v>22</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
         <v>24</v>
@@ -1322,10 +1334,10 @@
         <v>63</v>
       </c>
       <c r="O13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="P13" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="Q13" t="s">
         <v>29</v>
@@ -1333,28 +1345,28 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D14" t="s">
         <v>20</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="G14" t="s">
         <v>22</v>
       </c>
       <c r="H14" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I14" t="s">
         <v>24</v>
@@ -1372,10 +1384,10 @@
         <v>105</v>
       </c>
       <c r="O14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="P14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="Q14" t="s">
         <v>29</v>
@@ -1383,28 +1395,28 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
         <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
         <v>20</v>
       </c>
       <c r="E15" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F15" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G15" t="s">
         <v>22</v>
       </c>
       <c r="H15" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I15" t="s">
         <v>24</v>
@@ -1422,10 +1434,10 @@
         <v>141</v>
       </c>
       <c r="O15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="P15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="Q15" t="s">
         <v>29</v>
@@ -1433,19 +1445,19 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
         <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
         <v>20</v>
       </c>
       <c r="E16" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F16" t="s">
         <v>21</v>
@@ -1454,7 +1466,7 @@
         <v>22</v>
       </c>
       <c r="H16" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="I16" t="s">
         <v>24</v>
@@ -1472,10 +1484,10 @@
         <v>126</v>
       </c>
       <c r="O16" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="P16" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="Q16" t="s">
         <v>29</v>
@@ -1483,19 +1495,19 @@
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
         <v>20</v>
       </c>
       <c r="E17" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
         <v>21</v>
@@ -1504,7 +1516,7 @@
         <v>22</v>
       </c>
       <c r="H17" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I17" t="s">
         <v>24</v>
@@ -1522,10 +1534,10 @@
         <v>62</v>
       </c>
       <c r="O17" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="P17" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="Q17" t="s">
         <v>29</v>
@@ -1533,19 +1545,19 @@
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
         <v>18</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
         <v>20</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
         <v>21</v>
@@ -1554,7 +1566,7 @@
         <v>22</v>
       </c>
       <c r="H18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
@@ -1566,16 +1578,16 @@
         <v>80</v>
       </c>
       <c r="L18" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="N18">
         <v>16</v>
       </c>
       <c r="O18" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="P18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="Q18" t="s">
         <v>29</v>
@@ -1583,19 +1595,19 @@
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
         <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F19" t="s">
         <v>21</v>
@@ -1604,7 +1616,7 @@
         <v>22</v>
       </c>
       <c r="H19" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I19" t="s">
         <v>24</v>
@@ -1622,10 +1634,10 @@
         <v>21</v>
       </c>
       <c r="O19" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="P19" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="Q19" t="s">
         <v>29</v>
@@ -1633,19 +1645,19 @@
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B20" t="s">
         <v>18</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
         <v>21</v>
@@ -1654,7 +1666,7 @@
         <v>22</v>
       </c>
       <c r="H20" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I20" t="s">
         <v>24</v>
@@ -1672,10 +1684,10 @@
         <v>39</v>
       </c>
       <c r="O20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P20" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="Q20" t="s">
         <v>29</v>

</xml_diff>